<commit_message>
fix(review): Restore authentic logbook state, reframe FPR and noise sensitivity, and update bird-free audit as working hypothesis
</commit_message>
<xml_diff>
--- a/Tugas Akhir AS Ganjil 2026.xlsx
+++ b/Tugas Akhir AS Ganjil 2026.xlsx
@@ -15291,27 +15291,19 @@
       </c>
       <c r="G26" s="45" t="inlineStr">
         <is>
-          <t>60 menit</t>
+          <t>30 menit</t>
         </is>
       </c>
       <c r="H26" s="45" t="inlineStr">
         <is>
-          <t>1. Dataset: Membekukan dataset BirdCLEF+ 2026 yang terdiri dari 20 spesies burung Neotropis, total 4.351 klip audio (Galeri 3.653 klip, Query 200 klip tepat 10 per spesies, Kalibrasi 498 klip). Preprocessing audio dibekukan pada format 32 kHz mono, segmen 5.0 detik, dan normalisasi RMS 0.05.
+          <t>1. Dataset: Membekukan dataset BirdCLEF+ 2026 yang terdiri dari 20 spesies burung Neotropis, total 4.351 klip audio (Galeri 3.653 klip, Query 200 klip tepat 10 per spesies, Kalibrasi 498 klip). Preprocessing dibekukan pada 32 kHz mono, segmen 5.0 detik, dan normalisasi RMS 0.05.
 2. Partisi Bebas Kebocoran: Menerapkan Strict Recordist-Disjoint (Galeri 377 perekam, Query 68 perekam, Kalibrasi 95 perekam) dengan 0 overlap perekam antar-split (Zero Leakage).
-3. Pembanding (Representasi): Menyiapkan 4 representasi beku, yaitu R0 (MFCC 40-dim), R1 (Generic Audio Pretrained PANNs CNN14 2048-dim), R2 (Bioacoustic Pretrained BirdNET 1024-dim), dan R3 (Random Projection Control 1024-dim).
-4. Ukuran Keberhasilan: Menetapkan metrik mAP@10, kurva retensi performa relatif lintas level derau (Clean s/d -5 dB SNR), serta optimalisasi ambang batas Youden's J (tau*) untuk penolakan audio unknown open-set.</t>
-        </is>
-      </c>
-      <c r="I26" s="45" t="inlineStr">
-        <is>
-          <t>Pastikan partisi bebas kebocoran divalidasi dengan unit test otomatis sebelum memulai ekstraksi fitur.</t>
-        </is>
-      </c>
-      <c r="J26" s="45" t="inlineStr">
-        <is>
-          <t>Rencana eksperimen dan protokol pengukuran</t>
-        </is>
-      </c>
+3. Pembanding (Representasi): Menyiapkan 4 model pembanding beku, yaitu R0 (MFCC), R1 (Generic PANNs), R2 (Bioacoustic BirdNET), dan R3 (Random Control).
+4. Ukuran Keberhasilan: Menetapkan metrik mAP@10, kurva retensi performa relatif lintas level derau (Clean s/d -5 dB SNR), serta optimalisasi ambang batas Youden's J (tau*) untuk penolakan audio asing.</t>
+        </is>
+      </c>
+      <c r="I26" s="45" t="n"/>
+      <c r="J26" s="45" t="n"/>
       <c r="K26" s="46" t="inlineStr">
         <is>
           <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/data/manifests</t>
@@ -15345,52 +15337,20 @@
           <t>Rencana eksperimen dan protokol pengukuran</t>
         </is>
       </c>
-      <c r="E27" s="47" t="n">
-        <v>46276</v>
-      </c>
-      <c r="F27" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G27" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H27" s="45" t="inlineStr">
-        <is>
-          <t>Menyusun rancangan protokol eksperimental paired robustness untuk 5 eksperimen utama:
-- E1: Evaluasi retrieval kemiripan pada kondisi clean (baseline benchmarking).
-- E2: Uji ketahanan terhadap degradasi derau sintetis dan lingkungan ITERA pada tingkat SNR +20 dB s/d -5 dB.
-- E3: Kalibrasi dan pengujian ambang batas keterbukaan (Open-Set Thresholding tau*) dengan rasio 1:1.
-- E4: Pengujian sensitivitas profil derau soundscape BirdCLEF berpasangan (per-query paired analysis).
-- E5: Taksonomi analisis moda kegagalan retrieval berbasis batas ambang keterbukaan.
-Membekukan formula percampuran derau aditif berbasis kontrol daya sinyal kueri.</t>
-        </is>
-      </c>
-      <c r="I27" s="45" t="inlineStr">
-        <is>
-          <t>Pastikan protokol mixing derau konsisten pada seluruh representasi, dan pastikan split recordist-disjoint divalidasi dengan unit test otomatis.</t>
-        </is>
-      </c>
-      <c r="J27" s="45" t="inlineStr">
-        <is>
-          <t>Kesiapan data dan pipeline eksperimen (P4/P5)</t>
-        </is>
-      </c>
-      <c r="K27" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/Rencana-eksperimen-bimbingan/minggu-1</t>
-        </is>
-      </c>
+      <c r="E27" s="47" t="n"/>
+      <c r="F27" s="45" t="n"/>
+      <c r="G27" s="45" t="n"/>
+      <c r="H27" s="45" t="n"/>
+      <c r="I27" s="45" t="n"/>
+      <c r="J27" s="45" t="n"/>
+      <c r="K27" s="45" t="n"/>
       <c r="L27" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M27" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="54" customHeight="1" s="65">
@@ -15412,46 +15372,20 @@
           <t>Hasil pembanding pertama</t>
         </is>
       </c>
-      <c r="E28" s="47" t="n">
-        <v>46280</v>
-      </c>
-      <c r="F28" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G28" s="45" t="inlineStr">
-        <is>
-          <t>45 menit</t>
-        </is>
-      </c>
-      <c r="H28" s="45" t="inlineStr">
-        <is>
-          <t>Mengekstraksi embedding representasi baseline R0 (MFCC 40-dim) dan kontrol negatif R3 (Random Gaussian 1024-dim). Menjalankan retrieval similarity pada kondisi clean (E1) terhadap 200 query dan 3.653 galeri. Hasil terverifikasi: R0 menghasilkan mAP@10 = 0.1322, sedangkan kontrol acak R3 menghasilkan mAP@10 = 0.0519 (sesuai ekspektasi teoretis 1/20 = 0.05). Memvalidasi kalkulasi metrik mAP@10 dengan library scikit-learn dan rank correlation.</t>
-        </is>
-      </c>
-      <c r="I28" s="45" t="inlineStr">
-        <is>
-          <t>Siapkan integrasi arsitektur deep learning (PANNs CNN14 dan BirdNET) dan bandingkan performa clean retrieval sebelum masuk ke tahap derau.</t>
-        </is>
-      </c>
-      <c r="J28" s="45" t="inlineStr">
-        <is>
-          <t>Ekstraksi fitur deep learning dan persiapan pengujian clean retrieval (E1).</t>
-        </is>
-      </c>
-      <c r="K28" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E1_clean_retrieval</t>
-        </is>
-      </c>
+      <c r="E28" s="47" t="n"/>
+      <c r="F28" s="45" t="n"/>
+      <c r="G28" s="45" t="n"/>
+      <c r="H28" s="45" t="n"/>
+      <c r="I28" s="45" t="n"/>
+      <c r="J28" s="45" t="n"/>
+      <c r="K28" s="45" t="n"/>
       <c r="L28" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M28" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="54" customHeight="1" s="65">
@@ -15473,46 +15407,20 @@
           <t>Kesiapan data dan pipeline eksperimen</t>
         </is>
       </c>
-      <c r="E29" s="47" t="n">
-        <v>46283</v>
-      </c>
-      <c r="F29" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G29" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H29" s="45" t="inlineStr">
-        <is>
-          <t>Menyelesaikan pengambilan data derau lingkungan di ITERA menggunakan perekam AudioMoth (32 kHz). Mengunduh checkpoint pretrained CNN14 (Cnn14_mAP=0.431.pth) dan pretrained BirdNET. Membangun pipeline ekstraksi fitur offline otomatis berbasis batch processing PyTorch untuk mengekstrak seluruh galeri (3.653 berkas) dan kueri (200 berkas). Memverifikasi dimensi embedding (R0: 40-d, R1: 2048-d, R2: 1024-d, R3: 1024-d).</t>
-        </is>
-      </c>
-      <c r="I29" s="45" t="inlineStr">
-        <is>
-          <t>Pastikan kalibrasi level gain dan sampling rate AudioMoth sinkron dengan format dataset galeri (32 kHz) dan lakukan normalisasi L2 pada seluruh embedding.</t>
-        </is>
-      </c>
-      <c r="J29" s="45" t="inlineStr">
-        <is>
-          <t>Eksperimen utama gelombang pertama (E1 dan E2).</t>
-        </is>
-      </c>
-      <c r="K29" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/data/itera_noise</t>
-        </is>
-      </c>
+      <c r="E29" s="47" t="n"/>
+      <c r="F29" s="45" t="n"/>
+      <c r="G29" s="45" t="n"/>
+      <c r="H29" s="45" t="n"/>
+      <c r="I29" s="45" t="n"/>
+      <c r="J29" s="45" t="n"/>
+      <c r="K29" s="45" t="n"/>
       <c r="L29" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M29" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="54" customHeight="1" s="65">
@@ -15534,46 +15442,20 @@
           <t>Eksperimen utama, gelombang pertama</t>
         </is>
       </c>
-      <c r="E30" s="47" t="n">
-        <v>46287</v>
-      </c>
-      <c r="F30" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G30" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H30" s="45" t="inlineStr">
-        <is>
-          <t>Menuntaskan Eksperimen E1 (Clean Benchmark) dan E2 gelombang awal (SNR +20 dB s/d 0 dB). Pada kondisi Clean, R2 (BirdNET) mencapai keunggulan mutlak mAP@10 = 0.9169, disusul R1 (PANNs) = 0.4195, R0 (MFCC) = 0.1322, dan R3 = 0.0519. Menemukan stabilitas tinggi pada BirdNET pada derau ringan, sedangkan PANNs mulai terdegradasi saat SNR menurun ke 0 dB.</t>
-        </is>
-      </c>
-      <c r="I30" s="45" t="inlineStr">
-        <is>
-          <t>Lanjutkan injeksi derau hingga kondisi sangat ekstrem (-5 dB SNR) dan perluas variasi profil derau dari beberapa lokasi kampus.</t>
-        </is>
-      </c>
-      <c r="J30" s="45" t="inlineStr">
-        <is>
-          <t>Penyelesaian seluruh level derau E2 dan bank derau komprehensif.</t>
-        </is>
-      </c>
-      <c r="K30" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E2_noise_robustness</t>
-        </is>
-      </c>
+      <c r="E30" s="47" t="n"/>
+      <c r="F30" s="45" t="n"/>
+      <c r="G30" s="45" t="n"/>
+      <c r="H30" s="45" t="n"/>
+      <c r="I30" s="45" t="n"/>
+      <c r="J30" s="45" t="n"/>
+      <c r="K30" s="45" t="n"/>
       <c r="L30" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M30" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="54" customHeight="1" s="65">
@@ -15595,46 +15477,20 @@
           <t>Eksperimen utama, gelombang kedua</t>
         </is>
       </c>
-      <c r="E31" s="47" t="n">
-        <v>46291</v>
-      </c>
-      <c r="F31" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G31" s="45" t="inlineStr">
-        <is>
-          <t>90 menit</t>
-        </is>
-      </c>
-      <c r="H31" s="45" t="inlineStr">
-        <is>
-          <t>Menyelesaikan seluruh matriks pengujian E2 (20 kombinasi eksperimen, SNR +20 dB s/d -5 dB). Menemukan anomali penting: pada -5 dB, retensi BirdNET bertahan di 78.43% (mAP = 0.7191), sementara PANNs terdegradasi tajam ke mAP = 0.0590 (retensi 14.22%), berada di bawah retensi MFCC (26.42%, mAP = 0.0349). Menyelesaikan pengumpulan bank derau ITERA hingga 1.799 file dari 5 lokasi (Embung F, Gedung F, GKU 1, Kebun Raya, Masjid At-Tanwir).</t>
-        </is>
-      </c>
-      <c r="I31" s="45" t="inlineStr">
-        <is>
-          <t>Analisis secara mendalam mengapa representasi audio generic (PANNs) kalah tangguh dibandingkan representasi spesifik bioakustik pada derau ekstrem.</t>
-        </is>
-      </c>
-      <c r="J31" s="45" t="inlineStr">
-        <is>
-          <t>Eksperimen open-set calibration (E3).</t>
-        </is>
-      </c>
-      <c r="K31" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E2_noise_robustness</t>
-        </is>
-      </c>
+      <c r="E31" s="47" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="45" t="n"/>
+      <c r="H31" s="45" t="n"/>
+      <c r="I31" s="45" t="n"/>
+      <c r="J31" s="45" t="n"/>
+      <c r="K31" s="45" t="n"/>
       <c r="L31" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="54" customHeight="1" s="65">
@@ -15656,46 +15512,20 @@
           <t>Tinjauan hasil sementara dan koreksi arah</t>
         </is>
       </c>
-      <c r="E32" s="47" t="n">
-        <v>46295</v>
-      </c>
-      <c r="F32" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G32" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H32" s="45" t="inlineStr">
-        <is>
-          <t>Melaporkan hasil Eksperimen E3 (Open-Set Thresholding). Mengonstruksi split unknown kalibrasi (498 klip) dan unknown uji (200 klip) yang terisolasi dari takson target. Mengoptimalkan ambang batas Youden's J pada kalibrasi: R2 tau* = 0.7128 (J = 0.4779) dan R1 tau* = 0.9117. Menguji fenomena pergeseran titik operasi (H4): Pada kondisi derau ekstrem (-5 dB), recall BirdNET turun dari 86% ke 44.5% karena pelemahan kesamaan secara global, sedangkan FPR PANNs meledak hingga 81.5%.</t>
-        </is>
-      </c>
-      <c r="I32" s="45" t="inlineStr">
-        <is>
-          <t>Laporkan secara jujur bahwa pada kondisi clean, BirdNET menerima 39% derau ITERA karena adanya biofoni lokal pada trigger frekuensi di pohon. Hindari klaim penolakan derau mutlak.</t>
-        </is>
-      </c>
-      <c r="J32" s="45" t="inlineStr">
-        <is>
-          <t>Eksperimen E4 dan pengujian inferensi statistik bootstrap.</t>
-        </is>
-      </c>
-      <c r="K32" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E3_open_set_threshold</t>
-        </is>
-      </c>
+      <c r="E32" s="47" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="45" t="n"/>
+      <c r="I32" s="45" t="n"/>
+      <c r="J32" s="45" t="n"/>
+      <c r="K32" s="45" t="n"/>
       <c r="L32" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="54" customHeight="1" s="65">
@@ -15717,46 +15547,20 @@
           <t>Analisis hasil dan penyusunan tabel serta grafik</t>
         </is>
       </c>
-      <c r="E33" s="47" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F33" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G33" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H33" s="45" t="inlineStr">
-        <is>
-          <t>Melaksanakan Eksperimen E4 (Sensitivitas Profil Derau Soundscape) pada seluruh 4 representasi dengan paired per-query storage. Menjalankan inferensi statistik non-parametrik bootstrap (B=1000 resamples) untuk validasi formal: H1 (Retensi R2 vs R1: diff +0.6421, CI [0.559, 0.715], p &lt; 0.001, Terdukung), H2 (Retensi R2 vs R0: diff +0.5201, CI [0.447, 0.589], p &lt; 0.001, Terdukung), H3 ditandai 'Tidak Diuji (Deferred)' karena belum tersedianya anotasi soundscape in-situ terverifikasi. Membuat visualisasi kurva degradasi SNR, boxplot distribusi kesamaan, dan grafik retensi mAP.</t>
-        </is>
-      </c>
-      <c r="I33" s="45" t="inlineStr">
-        <is>
-          <t>Pastikan naskah mencatat secara jujur bahwa p = 0.6100 pada E4 bukan bukti ekuivalensi profil derau dan nyatakan batasan eksperimen aditif secara transparan.</t>
-        </is>
-      </c>
-      <c r="J33" s="45" t="inlineStr">
-        <is>
-          <t>Analisis moda kegagalan (E5) dan verifikasi keterulangan (P10).</t>
-        </is>
-      </c>
-      <c r="K33" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E4_real_soundscape</t>
-        </is>
-      </c>
+      <c r="E33" s="47" t="n"/>
+      <c r="F33" s="45" t="n"/>
+      <c r="G33" s="45" t="n"/>
+      <c r="H33" s="45" t="n"/>
+      <c r="I33" s="45" t="n"/>
+      <c r="J33" s="45" t="n"/>
+      <c r="K33" s="45" t="n"/>
       <c r="L33" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M33" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="54" customHeight="1" s="65">
@@ -15778,46 +15582,20 @@
           <t>Penutupan penelitian dan verifikasi keterulangan</t>
         </is>
       </c>
-      <c r="E34" s="47" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F34" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G34" s="45" t="inlineStr">
-        <is>
-          <t>45 menit</t>
-        </is>
-      </c>
-      <c r="H34" s="45" t="inlineStr">
-        <is>
-          <t>Menyelesaikan Eksperimen E5 (Taksonomi Moda Kegagalan) dengan random stratified sampling melintasi 16 takson burung beragam. Mengklasifikasikan 30 kasus kegagalan ke dalam 3 moda fisik: 11 Top-1 Confusion Above Tau (36.67%), 11 Open-Set False Rejection (36.67%), dan 8 Total Retrieval Collapse (26.67%). Mengunci seluruh manifes dataset dengan checksum SHA-256 dan memastikan test suite 9/9 PASS lolos secara konsisten di Windows/Linux/macOS.</t>
-        </is>
-      </c>
-      <c r="I34" s="45" t="inlineStr">
-        <is>
-          <t>Pastikan seluruh berkas di folder results/raw dan results/processed sinkron 100% tanpa adanya perbedaan desimal atau format.</t>
-        </is>
-      </c>
-      <c r="J34" s="45" t="inlineStr">
-        <is>
-          <t>Penyusunan kerangka naskah skripsi lengkap.</t>
-        </is>
-      </c>
-      <c r="K34" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/artifacts/reproducibility</t>
-        </is>
-      </c>
+      <c r="E34" s="47" t="n"/>
+      <c r="F34" s="45" t="n"/>
+      <c r="G34" s="45" t="n"/>
+      <c r="H34" s="45" t="n"/>
+      <c r="I34" s="45" t="n"/>
+      <c r="J34" s="45" t="n"/>
+      <c r="K34" s="45" t="n"/>
       <c r="L34" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M34" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="54" customHeight="1" s="65">
@@ -15839,46 +15617,20 @@
           <t>Kerangka naskah dan bab metode</t>
         </is>
       </c>
-      <c r="E35" s="47" t="n">
-        <v>46301</v>
-      </c>
-      <c r="F35" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G35" s="45" t="inlineStr">
-        <is>
-          <t>90 menit</t>
-        </is>
-      </c>
-      <c r="H35" s="45" t="inlineStr">
-        <is>
-          <t>Menyusun draf Bab 1 (Pendahuluan, 5 Research Questions, Batasan Masalah), Bab 2 (Tinjauan Pustaka Bioakustik, Ekstraksi Fitur Beku, Karakteristik Akustik Lingkungan Tropis), dan Bab 3 (Metodologi Penelitian, Desain Eksperimen E1-E5, Formulasi Matematis SNR mixing, mAP@10, Youden's J, ECE). Menegaskan rasionalisasi ilmiah mengapa fine-tuning dihindari dan representasi dievaluasi dalam kondisi beku (frozen zero-shot).</t>
-        </is>
-      </c>
-      <c r="I35" s="45" t="inlineStr">
-        <is>
-          <t>Perjelas justifikasi metodologis mengapa evaluasi paired per-query penting untuk mengontrol varians antar-sampel kicauan burung.</t>
-        </is>
-      </c>
-      <c r="J35" s="45" t="inlineStr">
-        <is>
-          <t>Penulisan Bab 4 (Hasil dan Pembahasan).</t>
-        </is>
-      </c>
-      <c r="K35" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/paper/manuscript.md</t>
-        </is>
-      </c>
+      <c r="E35" s="47" t="n"/>
+      <c r="F35" s="45" t="n"/>
+      <c r="G35" s="45" t="n"/>
+      <c r="H35" s="45" t="n"/>
+      <c r="I35" s="45" t="n"/>
+      <c r="J35" s="45" t="n"/>
+      <c r="K35" s="45" t="n"/>
       <c r="L35" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M35" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="54" customHeight="1" s="65">
@@ -15900,46 +15652,20 @@
           <t>Bab hasil dan pembahasan</t>
         </is>
       </c>
-      <c r="E36" s="47" t="n">
-        <v>46302</v>
-      </c>
-      <c r="F36" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G36" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H36" s="45" t="inlineStr">
-        <is>
-          <t>Menyusun Bab 4 (Hasil dan Pembahasan komprehensif E1 s/d E5). Memasukkan tabel signifikansi statistik bootstrap B=1000, pembahasan fenomena pergeseran titik operasi (H4), penjelasan anomali +20 dB PANNs sebagai observasi empiris yang belum terjelaskan, serta analisis akustik biofoni kanopi pohon pada bank derau ITERA yang menjelaskan angka FPR.</t>
-        </is>
-      </c>
-      <c r="I36" s="45" t="inlineStr">
-        <is>
-          <t>Koreksi narasi agar tidak mengklaim domain-invariance secara absolut dan pastikan seluruh angka di naskah cocok dengan data mentah.</t>
-        </is>
-      </c>
-      <c r="J36" s="45" t="inlineStr">
-        <is>
-          <t>Draf lengkap naskah skripsi dan ringkasan eksekutif (P13).</t>
-        </is>
-      </c>
-      <c r="K36" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/paper/manuscript.md</t>
-        </is>
-      </c>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="45" t="n"/>
+      <c r="G36" s="45" t="n"/>
+      <c r="H36" s="45" t="n"/>
+      <c r="I36" s="45" t="n"/>
+      <c r="J36" s="45" t="n"/>
+      <c r="K36" s="45" t="n"/>
       <c r="L36" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M36" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="54" customHeight="1" s="65">
@@ -15961,46 +15687,20 @@
           <t>Draf lengkap dan tinjauan menyeluruh</t>
         </is>
       </c>
-      <c r="E37" s="47" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F37" s="45" t="inlineStr">
-        <is>
-          <t>Luring</t>
-        </is>
-      </c>
-      <c r="G37" s="45" t="inlineStr">
-        <is>
-          <t>60 menit</t>
-        </is>
-      </c>
-      <c r="H37" s="45" t="inlineStr">
-        <is>
-          <t>Menuntaskan draf lengkap naskah skripsi (paper/manuscript.md), Panduan Komprehensif Tugas Akhir (dan ekspor PDF 97 KB), laporan keterulangan (reproducibility report), serta audit empiris biofoni derau ITERA. Melakukan sinkronisasi menyeluruh pada seluruh berkas dokumentasi experiments/ dan logbook bimbingan.</t>
-        </is>
-      </c>
-      <c r="I37" s="45" t="inlineStr">
-        <is>
-          <t>Periksa checklist artefak minimum dan pastikan seluruh tautan repositori aktif dan dapat diakses.</t>
-        </is>
-      </c>
-      <c r="J37" s="45" t="inlineStr">
-        <is>
-          <t>Finalisasi logbook dan kesiapan pendaftaran seminar hasil / sidang.</t>
-        </is>
-      </c>
-      <c r="K37" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/Panduan_Komprehensif_Tugas_Akhir.pdf</t>
-        </is>
-      </c>
+      <c r="E37" s="47" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="45" t="n"/>
+      <c r="I37" s="45" t="n"/>
+      <c r="J37" s="45" t="n"/>
+      <c r="K37" s="45" t="n"/>
       <c r="L37" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M37" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="54" customHeight="1" s="65">
@@ -16022,46 +15722,20 @@
           <t>Finalisasi dan kesiapan seminar atau sidang</t>
         </is>
       </c>
-      <c r="E38" s="47" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F38" s="45" t="inlineStr">
-        <is>
-          <t>Daring</t>
-        </is>
-      </c>
-      <c r="G38" s="45" t="inlineStr">
-        <is>
-          <t>45 menit</t>
-        </is>
-      </c>
-      <c r="H38" s="45" t="inlineStr">
-        <is>
-          <t>Menuntaskan seluruh perbaikan dari 5 temuan reviewer (sinkronisasi dokumen lama, standardisasi hash LF lintas platform, penulisan kesimpulan saintifik yang jujur pada E3/E4/E5, audit empiris biofoni derau ITERA, dan kelengkapan logbook P1-P14). Suite pengujian otomatis lolos 9/9 PASS (100%). Seluruh artefak minimum terverifikasi lengkap.</t>
-        </is>
-      </c>
-      <c r="I38" s="45" t="inlineStr">
-        <is>
-          <t>Logbook disetujui lengkap (14 pertemuan terpenuhi). Naskah dan artefak siap diajukan untuk pendaftaran Seminar Hasil / Ujian Skripsi.</t>
-        </is>
-      </c>
-      <c r="J38" s="45" t="inlineStr">
-        <is>
-          <t>Pendaftaran Seminar Hasil Tugas Akhir DSIC.</t>
-        </is>
-      </c>
-      <c r="K38" s="45" t="inlineStr">
-        <is>
-          <t>https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706</t>
-        </is>
-      </c>
+      <c r="E38" s="47" t="n"/>
+      <c r="F38" s="45" t="n"/>
+      <c r="G38" s="45" t="n"/>
+      <c r="H38" s="45" t="n"/>
+      <c r="I38" s="45" t="n"/>
+      <c r="J38" s="45" t="n"/>
+      <c r="K38" s="45" t="n"/>
       <c r="L38" s="45" t="inlineStr">
         <is>
-          <t>Selesai</t>
+          <t>Belum Dilaksanakan</t>
         </is>
       </c>
       <c r="M38" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -16104,8 +15778,8 @@
       </c>
       <c r="C43" s="46" t="inlineStr">
         <is>
-          <t>Naskah Skripsi: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/paper/manuscript.md 
-Panduan Komprehensif: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/Panduan_Komprehensif_Tugas_Akhir.md</t>
+          <t xml:space="preserve">Jurnal: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/jurnal
+Ringkasan Referensi: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/jurnal/referensi_jurnal_TA_bioakustik.csv </t>
         </is>
       </c>
       <c r="D43" s="48" t="b">
@@ -16123,8 +15797,8 @@
       </c>
       <c r="C44" s="46" t="inlineStr">
         <is>
-          <t>BirdCLEF+ 2026 Manifest: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/data/manifests 
-ITERA Noise Bank (1.799 audio): https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/data/itera_noise</t>
+          <t>Sumber: https://xeno-canto.org/explore/region  
+Dataset: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/data</t>
         </is>
       </c>
       <c r="D44" s="48" t="b">
@@ -16140,14 +15814,9 @@
           <t>Kode atau notebook eksperimen</t>
         </is>
       </c>
-      <c r="C45" s="45" t="inlineStr">
-        <is>
-          <t>Notebooks E1-E5: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/notebooks 
-Source Code: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/src</t>
-        </is>
-      </c>
+      <c r="C45" s="45" t="n"/>
       <c r="D45" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -16159,14 +15828,9 @@
           <t>Catatan konfigurasi dan langkah menjalankan ulang</t>
         </is>
       </c>
-      <c r="C46" s="45" t="inlineStr">
-        <is>
-          <t>Reproducibility Report: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/artifacts/reproducibility/reproducibility_report.md 
-Audit Derau ITERA: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/artifacts/reproducibility/bird_free_audit_report.md</t>
-        </is>
-      </c>
+      <c r="C46" s="45" t="n"/>
       <c r="D46" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -16178,14 +15842,9 @@
           <t>Hasil pembanding / baseline</t>
         </is>
       </c>
-      <c r="C47" s="45" t="inlineStr">
-        <is>
-          <t>Eksperimen E1 (Clean Benchmark): https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/experiments/E1_clean_retrieval 
-Raw Scores: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/results/raw/E1_clean_mAP.csv</t>
-        </is>
-      </c>
+      <c r="C47" s="45" t="n"/>
       <c r="D47" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -16197,14 +15856,9 @@
           <t>Hasil eksperimen utama</t>
         </is>
       </c>
-      <c r="C48" s="45" t="inlineStr">
-        <is>
-          <t>Processed Results &amp; Tables: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/results/processed 
-Raw Evaluation Logs: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/results/raw</t>
-        </is>
-      </c>
+      <c r="C48" s="45" t="n"/>
       <c r="D48" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -16216,14 +15870,9 @@
           <t>Tabel atau grafik yang menjawab pertanyaan penelitian</t>
         </is>
       </c>
-      <c r="C49" s="45" t="inlineStr">
-        <is>
-          <t>Hasil Gambar &amp; Grafik: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/results/figures 
-Tabel Ilmiah: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/tree/main/paper/tables</t>
-        </is>
-      </c>
+      <c r="C49" s="45" t="n"/>
       <c r="D49" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -16235,14 +15884,9 @@
           <t>Kesimpulan penelitian</t>
         </is>
       </c>
-      <c r="C50" s="45" t="inlineStr">
-        <is>
-          <t>Naskah Bab 5: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/paper/manuscript.md#5-kesimpulan-dan-saran 
-Ringkasan Hipotesis: https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/results/processed/statistical_significance_table.csv</t>
-        </is>
-      </c>
+      <c r="C50" s="45" t="n"/>
       <c r="D50" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -16254,14 +15898,9 @@
           <t>Draf skripsi atau draf artikel ilmiah</t>
         </is>
       </c>
-      <c r="C51" s="45" t="inlineStr">
-        <is>
-          <t>Naskah Lengkap (Markdown): https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/paper/manuscript.md 
-Panduan Komprehensif (PDF): https://github.com/Data-Systems-and-Intelligent-Computing/DSIC-2706/blob/main/Panduan_Komprehensif_Tugas_Akhir.pdf</t>
-        </is>
-      </c>
+      <c r="C51" s="45" t="n"/>
       <c r="D51" s="48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>